<commit_message>
Adiciona coluna de percentual de aulas cedidas no relatório
Nova coluna '% de aulas cedidas no semestre' = aulas cedidas ÷ aulas
programadas no semestre, mais a coluna intermediária 'Nº de aulas
programadas no semestre' para dar transparência ao cálculo.

Aulas programadas = nº de aulas semanais x nº de semanas letivas ativas
da turma (contado dia da semana por dia da semana, porque um feriado só
derruba o dia dele), da semana 1 até a data da última prova de 2ª
chamada confirmada pelo usuário (13/11 para turmas 10/12, que viajam
depois; 27/11 para turmas 9/11), descontando a semana vetada (conselho
de classe, tratada como zero aula por padrão).

Documentado na skill (novo item no Passo 0 pedindo essas datas à escola,
colunas atualizadas nos entregáveis) e os fatos concretos desta rodada em
referencia/estado_2sem_2026.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Relatorio_Tempos_Cedidos_Proposta_1.xlsx
+++ b/Horario desenvolvido/Relatorio_Tempos_Cedidos_Proposta_1.xlsx
@@ -17,14 +17,14 @@
     <sheet name="12C2" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'9C1'!$A$2:$D$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'9C2'!$A$2:$D$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'10C1'!$A$2:$D$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'10C2'!$A$2:$D$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'11C1'!$A$2:$D$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'11C2'!$A$2:$D$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'12C1'!$A$2:$D$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'12C2'!$A$2:$D$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'9C1'!$A$2:$F$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'9C2'!$A$2:$F$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'10C1'!$A$2:$F$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'10C2'!$A$2:$F$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'11C1'!$A$2:$F$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'11C2'!$A$2:$F$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'12C1'!$A$2:$F$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'12C2'!$A$2:$F$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -103,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -112,27 +114,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -500,13 +505,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,7 +541,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Nº de aulas programadas no semestre</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Nº de aulas cedidas para provas de outras disciplinas</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>% de aulas cedidas no semestre</t>
         </is>
       </c>
     </row>
@@ -549,11 +566,17 @@
           <t>BrSa (Bruno Vianna dos Santos)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>6</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.075</v>
       </c>
     </row>
     <row r="4">
@@ -567,11 +590,17 @@
           <t>Caro (Carolina Salles Kehl), SGa (Sabrina Gab), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>4</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.04210526315789474</v>
       </c>
     </row>
     <row r="5">
@@ -585,11 +614,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>2</v>
+      <c r="C5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.0625</v>
       </c>
     </row>
     <row r="6">
@@ -603,11 +638,17 @@
           <t>Caro (Carolina Salles Kehl), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>2</v>
+      <c r="D6" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="7">
@@ -621,11 +662,17 @@
           <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>2</v>
+      <c r="C7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="8">
@@ -639,11 +686,17 @@
           <t>Jana (Janaína Souza Silva)</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>2</v>
+      <c r="C8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.0625</v>
       </c>
     </row>
     <row r="9">
@@ -657,10 +710,16 @@
           <t>Caro (Carolina Salles Kehl)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="5" t="n">
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -675,10 +734,16 @@
           <t>FBri (Fábio Luís de Brito)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="8" t="n">
+      <c r="C10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -693,10 +758,16 @@
           <t>SMo (Samara Costa Moura)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="5" t="n">
+      <c r="C11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -711,10 +782,16 @@
           <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="8" t="n">
+      <c r="C12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -729,10 +806,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="5" t="n">
+      <c r="C13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -747,10 +830,16 @@
           <t>VSi (Vinícius de Paula Silveira)</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="8" t="n">
+      <c r="C14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -765,10 +854,16 @@
           <t>JuLa (Júlia Soares Leite Lanzarini de Carvalho)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" s="5" t="n">
+      <c r="C15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -783,10 +878,16 @@
           <t>APa (Ana Patricia Machado de Pinho Garcia), PaH (Paulo Henrique Sá Júnior), Velo (Rodrigo Veloso)</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -801,10 +902,16 @@
           <t>Fab (Fabio Merçon)</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="5" t="n">
+      <c r="C17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -819,10 +926,16 @@
           <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -837,10 +950,16 @@
           <t>DiS (Diana Lacs Sichel)</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="5" t="n">
+      <c r="C19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -855,10 +974,16 @@
           <t>SJu (Sérgio Luis Araújo Lopes Júnior)</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="8" t="n">
+      <c r="C20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -868,16 +993,22 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n">
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="9" t="n">
+        <v>617</v>
+      </c>
+      <c r="E21" s="9" t="n">
         <v>18</v>
       </c>
+      <c r="F21" s="11" t="n">
+        <v>0.02917341977309562</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D21"/>
+  <autoFilter ref="A2:F21"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -889,13 +1020,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -923,7 +1056,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Nº de aulas programadas no semestre</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Nº de aulas cedidas para provas de outras disciplinas</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>% de aulas cedidas no semestre</t>
         </is>
       </c>
     </row>
@@ -938,11 +1081,17 @@
           <t>Caro (Carolina Salles Kehl), SGa (Sabrina Gab), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>4</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.04210526315789474</v>
       </c>
     </row>
     <row r="4">
@@ -956,11 +1105,17 @@
           <t>Jana (Janaína Souza Silva)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="8" t="n">
+      <c r="C4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>4</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.125</v>
       </c>
     </row>
     <row r="5">
@@ -974,11 +1129,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>2</v>
+      <c r="C5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.0625</v>
       </c>
     </row>
     <row r="6">
@@ -992,11 +1153,17 @@
           <t>Caro (Carolina Salles Kehl), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>2</v>
+      <c r="D6" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="7">
@@ -1010,11 +1177,17 @@
           <t>BrSa (Bruno Vianna dos Santos)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D7" s="5" t="n">
-        <v>2</v>
+      <c r="D7" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.025</v>
       </c>
     </row>
     <row r="8">
@@ -1028,11 +1201,17 @@
           <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>1</v>
+      <c r="D8" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="9">
@@ -1046,10 +1225,16 @@
           <t>Caro (Carolina Salles Kehl)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="5" t="n">
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1064,10 +1249,16 @@
           <t>FBri (Fábio Luís de Brito)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="8" t="n">
+      <c r="C10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1082,10 +1273,16 @@
           <t>SMo (Samara Costa Moura)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="5" t="n">
+      <c r="C11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1100,10 +1297,16 @@
           <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="8" t="n">
+      <c r="C12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1118,10 +1321,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="5" t="n">
+      <c r="C13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1136,10 +1345,16 @@
           <t>VSi (Vinícius de Paula Silveira)</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="8" t="n">
+      <c r="C14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1154,10 +1369,16 @@
           <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" s="5" t="n">
+      <c r="C15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1172,10 +1393,16 @@
           <t>JuLa (Júlia Soares Leite Lanzarini de Carvalho)</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="8" t="n">
+      <c r="C16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1190,10 +1417,16 @@
           <t>APa (Ana Patricia Machado de Pinho Garcia), PaH (Paulo Henrique Sá Júnior), Velo (Rodrigo Veloso)</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1208,10 +1441,16 @@
           <t>Fab (Fabio Merçon)</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="8" t="n">
+      <c r="C18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1226,10 +1465,16 @@
           <t>DiS (Diana Lacs Sichel)</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="5" t="n">
+      <c r="C19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1244,10 +1489,16 @@
           <t>Tac (Taciana Novello Gatto)</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="8" t="n">
+      <c r="C20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1257,16 +1508,22 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n">
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="9" t="n">
+        <v>617</v>
+      </c>
+      <c r="E21" s="9" t="n">
         <v>15</v>
       </c>
+      <c r="F21" s="11" t="n">
+        <v>0.02431118314424635</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D21"/>
+  <autoFilter ref="A2:F21"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1278,13 +1535,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1312,7 +1571,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Nº de aulas programadas no semestre</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Nº de aulas cedidas para provas de outras disciplinas</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>% de aulas cedidas no semestre</t>
         </is>
       </c>
     </row>
@@ -1327,11 +1596,17 @@
           <t>APa (Ana Patricia Machado de Pinho Garcia)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>10</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.1851851851851852</v>
       </c>
     </row>
     <row r="4">
@@ -1345,11 +1620,17 @@
           <t>Eth (Ethel Vera Figur Driesen), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Swa (Greta Schwankhaus Oliveira)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>7</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.1029411764705882</v>
       </c>
     </row>
     <row r="5">
@@ -1363,11 +1644,17 @@
           <t>VSi (Vinícius de Paula Silveira)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="5" t="n">
+      <c r="C5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>4</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.1538461538461539</v>
       </c>
     </row>
     <row r="6">
@@ -1381,11 +1668,17 @@
           <t>EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Car (Carina Campagnani), Swa (Greta Schwankhaus Oliveira)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>2</v>
+      <c r="C6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="7">
@@ -1399,11 +1692,17 @@
           <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>2</v>
+      <c r="C7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="8">
@@ -1417,11 +1716,17 @@
           <t>ALu (Ana Lúcia Fonseca de Castro)</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>1</v>
+      <c r="C8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.03571428571428571</v>
       </c>
     </row>
     <row r="9">
@@ -1435,11 +1740,17 @@
           <t>BrSa (Bruno Vianna dos Santos)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="5" t="n">
-        <v>1</v>
+      <c r="D9" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.02380952380952381</v>
       </c>
     </row>
     <row r="10">
@@ -1453,11 +1764,17 @@
           <t>FBri (Fábio Luís de Brito)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>1</v>
+      <c r="C10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0.03846153846153846</v>
       </c>
     </row>
     <row r="11">
@@ -1471,10 +1788,16 @@
           <t>SGa (Sabrina Gab)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="5" t="n">
+      <c r="C11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1489,10 +1812,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="8" t="n">
+      <c r="C12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1507,10 +1836,16 @@
           <t>Lza (Luiza Maria Abreu de Mattos)</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1525,10 +1860,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="8" t="n">
+      <c r="C14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1543,10 +1884,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="5" t="n">
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1561,10 +1908,16 @@
           <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="8" t="n">
+      <c r="C16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1579,10 +1932,16 @@
           <t>Mlo (Marcelo Rios Lopes)</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="5" t="n">
+      <c r="C17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1597,10 +1956,16 @@
           <t>Mlo (Marcelo Rios Lopes)</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="8" t="n">
+      <c r="C18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1615,10 +1980,16 @@
           <t>SMo (Samara Costa Moura)</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="5" t="n">
+      <c r="C19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1633,10 +2004,16 @@
           <t>MFo (Mário Henrique Fonseca)</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D20" s="8" t="n">
+      <c r="C20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1651,10 +2028,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C21" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="5" t="n">
+      <c r="C21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1669,10 +2052,16 @@
           <t>BPad (Beatriz de Matos Ferreira Padrão)</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" s="8" t="n">
+      <c r="C22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1687,10 +2076,16 @@
           <t>Kle (André Luiz Medeiros Klevenhusen)</t>
         </is>
       </c>
-      <c r="C23" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="5" t="n">
+      <c r="C23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1705,10 +2100,16 @@
           <t>SJu (Sérgio Luis Araújo Lopes Júnior)</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="8" t="n">
+      <c r="C24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1718,16 +2119,22 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="10" t="n"/>
-      <c r="D25" s="10" t="n">
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="9" t="n"/>
+      <c r="D25" s="9" t="n">
+        <v>598</v>
+      </c>
+      <c r="E25" s="9" t="n">
         <v>28</v>
       </c>
+      <c r="F25" s="11" t="n">
+        <v>0.04682274247491638</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D25"/>
+  <autoFilter ref="A2:F25"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1739,13 +2146,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1773,7 +2182,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Nº de aulas programadas no semestre</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Nº de aulas cedidas para provas de outras disciplinas</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>% de aulas cedidas no semestre</t>
         </is>
       </c>
     </row>
@@ -1788,11 +2207,17 @@
           <t>Eth (Ethel Vera Figur Driesen), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Swa (Greta Schwankhaus Oliveira)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>7</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.1029411764705882</v>
       </c>
     </row>
     <row r="4">
@@ -1806,11 +2231,17 @@
           <t>MFo (Mário Henrique Fonseca)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="8" t="n">
+      <c r="C4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>5</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.1923076923076923</v>
       </c>
     </row>
     <row r="5">
@@ -1824,11 +2255,17 @@
           <t>Mlo (Marcelo Rios Lopes)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="5" t="n">
+      <c r="C5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>3</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.1071428571428571</v>
       </c>
     </row>
     <row r="6">
@@ -1842,11 +2279,17 @@
           <t>BPad (Beatriz de Matos Ferreira Padrão)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="8" t="n">
+      <c r="C6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>3</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.1153846153846154</v>
       </c>
     </row>
     <row r="7">
@@ -1860,11 +2303,17 @@
           <t>EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Car (Carina Campagnani), Swa (Greta Schwankhaus Oliveira)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>2</v>
+      <c r="C7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="8">
@@ -1878,11 +2327,17 @@
           <t>ALu (Ana Lúcia Fonseca de Castro)</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>2</v>
+      <c r="C8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="9">
@@ -1896,11 +2351,17 @@
           <t>Vir (Virgínia Granadeiro Chaves Silva)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="5" t="n">
-        <v>2</v>
+      <c r="D9" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.03571428571428571</v>
       </c>
     </row>
     <row r="10">
@@ -1914,11 +2375,17 @@
           <t>BrSa (Bruno Vianna dos Santos)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="8" t="n">
-        <v>2</v>
+      <c r="D10" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="11">
@@ -1932,11 +2399,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>1</v>
+      <c r="C11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.03571428571428571</v>
       </c>
     </row>
     <row r="12">
@@ -1950,11 +2423,17 @@
           <t>FBri (Fábio Luís de Brito)</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>1</v>
+      <c r="C12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>0.03846153846153846</v>
       </c>
     </row>
     <row r="13">
@@ -1968,11 +2447,17 @@
           <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>1</v>
+      <c r="C13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0.03846153846153846</v>
       </c>
     </row>
     <row r="14">
@@ -1986,10 +2471,16 @@
           <t>SGa (Sabrina Gab)</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="8" t="n">
+      <c r="C14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2004,10 +2495,16 @@
           <t>Lza (Luiza Maria Abreu de Mattos)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2022,10 +2519,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="8" t="n">
+      <c r="C16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2040,10 +2543,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="5" t="n">
+      <c r="C17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2058,10 +2567,16 @@
           <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="8" t="n">
+      <c r="C18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2076,10 +2591,16 @@
           <t>Mlo (Marcelo Rios Lopes)</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="5" t="n">
+      <c r="C19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2094,10 +2615,16 @@
           <t>VSi (Vinícius de Paula Silveira)</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D20" s="8" t="n">
+      <c r="C20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2112,10 +2639,16 @@
           <t>SMo (Samara Costa Moura)</t>
         </is>
       </c>
-      <c r="C21" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="5" t="n">
+      <c r="C21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2130,10 +2663,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" s="8" t="n">
+      <c r="C22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2148,10 +2687,16 @@
           <t>Kle (André Luiz Medeiros Klevenhusen)</t>
         </is>
       </c>
-      <c r="C23" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="5" t="n">
+      <c r="C23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2166,10 +2711,16 @@
           <t>Tac (Taciana Novello Gatto)</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="8" t="n">
+      <c r="C24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2179,16 +2730,22 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="10" t="n"/>
-      <c r="D25" s="10" t="n">
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="9" t="n"/>
+      <c r="D25" s="9" t="n">
+        <v>598</v>
+      </c>
+      <c r="E25" s="9" t="n">
         <v>29</v>
       </c>
+      <c r="F25" s="11" t="n">
+        <v>0.04849498327759198</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D25"/>
+  <autoFilter ref="A2:F25"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2200,13 +2757,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2234,7 +2793,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Nº de aulas programadas no semestre</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Nº de aulas cedidas para provas de outras disciplinas</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>% de aulas cedidas no semestre</t>
         </is>
       </c>
     </row>
@@ -2249,11 +2818,17 @@
           <t>ClaMe (Clarissa Duarte Loureiro de Melo)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>8</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.1739130434782609</v>
       </c>
     </row>
     <row r="4">
@@ -2267,11 +2842,17 @@
           <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="8" t="n">
+      <c r="C4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>4</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.1379310344827586</v>
       </c>
     </row>
     <row r="5">
@@ -2285,11 +2866,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="5" t="n">
-        <v>2</v>
+      <c r="D5" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.03174603174603174</v>
       </c>
     </row>
     <row r="6">
@@ -2303,11 +2890,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>2</v>
+      <c r="C6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.0625</v>
       </c>
     </row>
     <row r="7">
@@ -2321,11 +2914,17 @@
           <t>Ver (Verena Alberti)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="5" t="n">
-        <v>2</v>
+      <c r="D7" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.04166666666666666</v>
       </c>
     </row>
     <row r="8">
@@ -2339,11 +2938,17 @@
           <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>2</v>
+      <c r="C8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.06451612903225806</v>
       </c>
     </row>
     <row r="9">
@@ -2357,11 +2962,17 @@
           <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>2</v>
+      <c r="C9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="10">
@@ -2375,11 +2986,17 @@
           <t>Cadu (Carlos Eduardo Lima)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="8" t="n">
-        <v>1</v>
+      <c r="D10" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0.02083333333333333</v>
       </c>
     </row>
     <row r="11">
@@ -2393,11 +3010,17 @@
           <t>JJ (João Jorge Fernandes Chaves)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>1</v>
+      <c r="C11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.03125</v>
       </c>
     </row>
     <row r="12">
@@ -2411,10 +3034,16 @@
           <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2429,10 +3058,16 @@
           <t>CBu (Claudia Burkhardt), SGa (Sabrina Gab), Swa (Greta Schwankhaus Oliveira)</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2447,10 +3082,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="8" t="n">
+      <c r="C14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2465,10 +3106,16 @@
           <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="5" t="n">
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2483,10 +3130,16 @@
           <t>CBu (Claudia Burkhardt), Swa (Greta Schwankhaus Oliveira), SGa (Sabrina Gab)</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="8" t="n">
+      <c r="C16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2501,10 +3154,16 @@
           <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="5" t="n">
+      <c r="C17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2519,10 +3178,16 @@
           <t>Bea (Beatriz Souza Andrade Maciel)</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2537,10 +3202,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="5" t="n">
+      <c r="D19" s="3" t="n">
+        <v>126</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2555,10 +3226,16 @@
           <t>APa (Ana Patricia Machado de Pinho Garcia)</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D20" s="8" t="n">
+      <c r="C20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2573,10 +3250,16 @@
           <t>ACo (Alexandre Braga Badaue Coelho)</t>
         </is>
       </c>
-      <c r="C21" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="5" t="n">
+      <c r="C21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2591,10 +3274,16 @@
           <t>Kle (André Luiz Medeiros Klevenhusen)</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="8" t="n">
+      <c r="C22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2604,16 +3293,22 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n">
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="9" t="n"/>
+      <c r="D23" s="9" t="n">
+        <v>837</v>
+      </c>
+      <c r="E23" s="9" t="n">
         <v>24</v>
       </c>
+      <c r="F23" s="11" t="n">
+        <v>0.02867383512544803</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D23"/>
+  <autoFilter ref="A2:F23"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2625,13 +3320,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2659,7 +3356,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Nº de aulas programadas no semestre</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Nº de aulas cedidas para provas de outras disciplinas</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>% de aulas cedidas no semestre</t>
         </is>
       </c>
     </row>
@@ -2674,11 +3381,17 @@
           <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>7</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.1555555555555556</v>
       </c>
     </row>
     <row r="4">
@@ -2692,11 +3405,17 @@
           <t>JJ (João Jorge Fernandes Chaves)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="8" t="n">
+      <c r="C4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>5</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.15625</v>
       </c>
     </row>
     <row r="5">
@@ -2710,11 +3429,17 @@
           <t>ClaMe (Clarissa Duarte Loureiro de Melo)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>4</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.08888888888888889</v>
       </c>
     </row>
     <row r="6">
@@ -2728,11 +3453,17 @@
           <t>PaH (Paulo Henrique Sá Júnior)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>3</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="7">
@@ -2746,11 +3477,17 @@
           <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="5" t="n">
+      <c r="C7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>3</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.09375</v>
       </c>
     </row>
     <row r="8">
@@ -2764,11 +3501,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>2</v>
+      <c r="D8" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.03174603174603174</v>
       </c>
     </row>
     <row r="9">
@@ -2782,11 +3525,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>2</v>
+      <c r="C9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.0625</v>
       </c>
     </row>
     <row r="10">
@@ -2800,11 +3549,17 @@
           <t>ACo (Alexandre Braga Badaue Coelho)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>2</v>
+      <c r="C10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="11">
@@ -2818,11 +3573,17 @@
           <t>CBu (Claudia Burkhardt), Swa (Greta Schwankhaus Oliveira), SGa (Sabrina Gab)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>1</v>
+      <c r="C11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="12">
@@ -2836,11 +3597,17 @@
           <t>Ver (Verena Alberti)</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="8" t="n">
-        <v>1</v>
+      <c r="D12" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>0.02083333333333333</v>
       </c>
     </row>
     <row r="13">
@@ -2854,10 +3621,16 @@
           <t>CBu (Claudia Burkhardt), SGa (Sabrina Gab), Swa (Greta Schwankhaus Oliveira)</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2872,10 +3645,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="8" t="n">
+      <c r="C14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2890,10 +3669,16 @@
           <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="5" t="n">
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2908,10 +3693,16 @@
           <t>Cadu (Carlos Eduardo Lima)</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2926,10 +3717,16 @@
           <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="5" t="n">
+      <c r="C17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2944,10 +3741,16 @@
           <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="8" t="n">
+      <c r="C18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2962,10 +3765,16 @@
           <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" s="5" t="n">
+      <c r="C19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2980,10 +3789,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="D20" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2998,10 +3813,16 @@
           <t>APa (Ana Patricia Machado de Pinho Garcia)</t>
         </is>
       </c>
-      <c r="C21" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="5" t="n">
+      <c r="C21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3016,10 +3837,16 @@
           <t>Kle (André Luiz Medeiros Klevenhusen)</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="8" t="n">
+      <c r="C22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3029,16 +3856,22 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n">
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="9" t="n"/>
+      <c r="D23" s="9" t="n">
+        <v>837</v>
+      </c>
+      <c r="E23" s="9" t="n">
         <v>30</v>
       </c>
+      <c r="F23" s="11" t="n">
+        <v>0.03584229390681003</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D23"/>
+  <autoFilter ref="A2:F23"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3050,13 +3883,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3084,7 +3919,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Nº de aulas programadas no semestre</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Nº de aulas cedidas para provas de outras disciplinas</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>% de aulas cedidas no semestre</t>
         </is>
       </c>
     </row>
@@ -3099,11 +3944,17 @@
           <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>5</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.131578947368421</v>
       </c>
     </row>
     <row r="4">
@@ -3117,11 +3968,17 @@
           <t>Fab (Fabio Merçon)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="8" t="n">
+      <c r="C4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>5</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.1785714285714286</v>
       </c>
     </row>
     <row r="5">
@@ -3135,11 +3992,17 @@
           <t>Cadu (Carlos Eduardo Lima)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="5" t="n">
+      <c r="C5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>3</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.1071428571428571</v>
       </c>
     </row>
     <row r="6">
@@ -3153,11 +4016,17 @@
           <t>Deb (Debora Borba Linhares)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>3</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.05357142857142857</v>
       </c>
     </row>
     <row r="7">
@@ -3171,11 +4040,17 @@
           <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="5" t="n">
+      <c r="C7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>3</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.1071428571428571</v>
       </c>
     </row>
     <row r="8">
@@ -3189,11 +4064,17 @@
           <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>2</v>
+      <c r="D8" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="9">
@@ -3207,11 +4088,17 @@
           <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="5" t="n">
-        <v>2</v>
+      <c r="D9" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.02941176470588235</v>
       </c>
     </row>
     <row r="10">
@@ -3225,11 +4112,17 @@
           <t>Wag (Wagner Pinto da Silva)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="8" t="n">
-        <v>2</v>
+      <c r="D10" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="11">
@@ -3243,11 +4136,17 @@
           <t>PaH (Paulo Henrique Sá Júnior)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="5" t="n">
-        <v>2</v>
+      <c r="D11" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.05263157894736842</v>
       </c>
     </row>
     <row r="12">
@@ -3261,11 +4160,17 @@
           <t>Bre (Carlos Luiz Silva Brener)</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>2</v>
+      <c r="C12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="13">
@@ -3279,10 +4184,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3297,10 +4208,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="8" t="n">
+      <c r="C14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3315,10 +4232,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" s="5" t="n">
+      <c r="C15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3333,10 +4256,16 @@
           <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="8" t="n">
+      <c r="C16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3351,10 +4280,16 @@
           <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="5" t="n">
+      <c r="C17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3369,10 +4304,16 @@
           <t>JJ (João Jorge Fernandes Chaves)</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="8" t="n">
+      <c r="C18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3387,10 +4328,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="5" t="n">
+      <c r="D19" s="3" t="n">
+        <v>108</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3405,10 +4352,16 @@
           <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="8" t="n">
+      <c r="C20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3423,10 +4376,16 @@
           <t>Kle (André Luiz Medeiros Klevenhusen)</t>
         </is>
       </c>
-      <c r="C21" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="5" t="n">
+      <c r="C21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3436,16 +4395,22 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n">
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n">
+        <v>710</v>
+      </c>
+      <c r="E22" s="9" t="n">
         <v>29</v>
       </c>
+      <c r="F22" s="11" t="n">
+        <v>0.04084507042253521</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D22"/>
+  <autoFilter ref="A2:F22"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3457,13 +4422,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3491,7 +4458,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Nº de aulas programadas no semestre</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Nº de aulas cedidas para provas de outras disciplinas</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>% de aulas cedidas no semestre</t>
         </is>
       </c>
     </row>
@@ -3506,11 +4483,17 @@
           <t>Deb (Debora Borba Linhares)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>7</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.125</v>
       </c>
     </row>
     <row r="4">
@@ -3524,11 +4507,17 @@
           <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>4</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.05882352941176471</v>
       </c>
     </row>
     <row r="5">
@@ -3542,11 +4531,17 @@
           <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="5" t="n">
+      <c r="C5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>3</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.1071428571428571</v>
       </c>
     </row>
     <row r="6">
@@ -3560,11 +4555,17 @@
           <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>2</v>
+      <c r="D6" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="7">
@@ -3578,11 +4579,17 @@
           <t>Wag (Wagner Pinto da Silva)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="5" t="n">
-        <v>2</v>
+      <c r="D7" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="8">
@@ -3596,11 +4603,17 @@
           <t>Isb (Isabela Gomes Bustamante)</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>2</v>
+      <c r="D8" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.05263157894736842</v>
       </c>
     </row>
     <row r="9">
@@ -3614,11 +4627,17 @@
           <t>Fab (Fabio Merçon)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>1</v>
+      <c r="C9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.03571428571428571</v>
       </c>
     </row>
     <row r="10">
@@ -3632,10 +4651,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3650,10 +4675,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="5" t="n">
+      <c r="C11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3668,10 +4699,16 @@
           <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3686,10 +4723,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="5" t="n">
+      <c r="C13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3704,10 +4747,16 @@
           <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="8" t="n">
+      <c r="C14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3722,10 +4771,16 @@
           <t>Cadu (Carlos Eduardo Lima)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" s="5" t="n">
+      <c r="C15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3740,10 +4795,16 @@
           <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="8" t="n">
+      <c r="C16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3758,10 +4819,16 @@
           <t>Bre (Carlos Luiz Silva Brener)</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="5" t="n">
+      <c r="C17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3776,10 +4843,16 @@
           <t>JJ (João Jorge Fernandes Chaves)</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="8" t="n">
+      <c r="C18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3794,10 +4867,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="5" t="n">
+      <c r="D19" s="3" t="n">
+        <v>108</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3812,10 +4891,16 @@
           <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="8" t="n">
+      <c r="C20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3830,10 +4915,16 @@
           <t>Kle (André Luiz Medeiros Klevenhusen)</t>
         </is>
       </c>
-      <c r="C21" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="5" t="n">
+      <c r="C21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3843,16 +4934,22 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n">
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n">
+        <v>710</v>
+      </c>
+      <c r="E22" s="9" t="n">
         <v>21</v>
       </c>
+      <c r="F22" s="11" t="n">
+        <v>0.02957746478873239</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D22"/>
+  <autoFilter ref="A2:F22"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>